<commit_message>
docs: rbac-role-matrix.xlsx を dev の実データから再生成
user_permission_summary ビュー経由に切り替えた tools/rbac-matrix で作り直し。
前回生成から アプリ一覧（一般カテゴリ CM01〜CM03 等）・ロール数・ホスト名
（app-dev.ckk-tool.co.jp）が変わっていたぶんが反映される。

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_docs/rbac-role-matrix.xlsx
+++ b/_docs/rbac-role-matrix.xlsx
@@ -656,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -785,7 +785,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -810,7 +810,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -860,7 +860,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -906,11 +906,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>受注明細・指示書・工程実行・在庫</t>
+          <t>受注明細・指示書・工程実行・在庫・設計依頼</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1060,7 +1060,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1110,9 +1110,184 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E18" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>kiosk_approver</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>端末運用（承認）</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>端末とカードの特権操作を承認する。**自分では実行できない**</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>kiosk_operator</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>端末運用（申請）</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>共有端末とQRカードの面倒を見る。PIN の開示・端末の登録・カードの発行は申請して承認を受ける</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>4</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>privileged_approver</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>特権操作（承認）</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>特権操作の申請を承認・差し戻しできる。**自分では実行できない**（申請側の権限を持たない）</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>privileged_operator</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>特権操作（申請）</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>端末の秘密・端末アクセス・QRカード・個人データ・ユーザー変更を申請できる。実行は承認と期限の範囲内</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>7</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>security_auditor</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>監査（履歴閲覧）</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ログイン履歴・操作履歴を調べる。詳細と横断検索は申請して承認を受ける</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>user_approver</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ユーザー運用（承認）</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ユーザーの変更依頼と個人データ閲覧を承認する。**自分では実行できない**</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>user_operator</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ユーザー運用（申請）</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>入退社に伴うアカウント運用。利用停止・復帰・所属拠点の変更は変更依頼を出して承認を受ける</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
         <is>
           <t>○</t>
         </is>
@@ -1129,7 +1304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S19"/>
+  <dimension ref="A1:Z28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1151,6 +1326,13 @@
     <col width="15" customWidth="1" min="17" max="17"/>
     <col width="15" customWidth="1" min="18" max="18"/>
     <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="15" customWidth="1" min="21" max="21"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="23" max="23"/>
+    <col width="15" customWidth="1" min="24" max="24"/>
+    <col width="15" customWidth="1" min="25" max="25"/>
+    <col width="15" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1266,6 +1448,48 @@
 (staff)</t>
         </is>
       </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>端末運用（承認）
+(kiosk_approver)</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>端末運用（申請）
+(kiosk_operator)</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>特権操作（承認）
+(privileged_approver)</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>特権操作（申請）
+(privileged_operator)</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>監査（履歴閲覧）
+(security_auditor)</t>
+        </is>
+      </c>
+      <c r="Y1" s="4" t="inlineStr">
+        <is>
+          <t>ユーザー運用（承認）
+(user_approver)</t>
+        </is>
+      </c>
+      <c r="Z1" s="4" t="inlineStr">
+        <is>
+          <t>ユーザー運用（申請）
+(user_operator)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -1276,7 +1500,7 @@
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>SA01 試算
+          <t>SA01 価格試算
 SA02 価格表</t>
         </is>
       </c>
@@ -1349,6 +1573,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T2" s="8" t="inlineStr"/>
+      <c r="U2" s="8" t="inlineStr"/>
+      <c r="V2" s="8" t="inlineStr"/>
+      <c r="W2" s="8" t="inlineStr"/>
+      <c r="X2" s="8" t="inlineStr"/>
+      <c r="Y2" s="8" t="inlineStr"/>
+      <c r="Z2" s="8" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -1431,6 +1662,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T3" s="8" t="inlineStr"/>
+      <c r="U3" s="8" t="inlineStr"/>
+      <c r="V3" s="8" t="inlineStr"/>
+      <c r="W3" s="8" t="inlineStr"/>
+      <c r="X3" s="8" t="inlineStr"/>
+      <c r="Y3" s="8" t="inlineStr"/>
+      <c r="Z3" s="8" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1526,6 +1764,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T4" s="8" t="inlineStr"/>
+      <c r="U4" s="8" t="inlineStr"/>
+      <c r="V4" s="8" t="inlineStr"/>
+      <c r="W4" s="8" t="inlineStr"/>
+      <c r="X4" s="8" t="inlineStr"/>
+      <c r="Y4" s="8" t="inlineStr"/>
+      <c r="Z4" s="8" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -1575,7 +1820,11 @@
           <t>R</t>
         </is>
       </c>
-      <c r="K5" s="8" t="inlineStr"/>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
       <c r="L5" s="8" t="inlineStr">
         <is>
           <t>R</t>
@@ -1604,6 +1853,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T5" s="8" t="inlineStr"/>
+      <c r="U5" s="8" t="inlineStr"/>
+      <c r="V5" s="8" t="inlineStr"/>
+      <c r="W5" s="8" t="inlineStr"/>
+      <c r="X5" s="8" t="inlineStr"/>
+      <c r="Y5" s="8" t="inlineStr"/>
+      <c r="Z5" s="8" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1679,6 +1935,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T6" s="8" t="inlineStr"/>
+      <c r="U6" s="8" t="inlineStr"/>
+      <c r="V6" s="8" t="inlineStr"/>
+      <c r="W6" s="8" t="inlineStr"/>
+      <c r="X6" s="8" t="inlineStr"/>
+      <c r="Y6" s="8" t="inlineStr"/>
+      <c r="Z6" s="8" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -1753,6 +2016,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T7" s="8" t="inlineStr"/>
+      <c r="U7" s="8" t="inlineStr"/>
+      <c r="V7" s="8" t="inlineStr"/>
+      <c r="W7" s="8" t="inlineStr"/>
+      <c r="X7" s="8" t="inlineStr"/>
+      <c r="Y7" s="8" t="inlineStr"/>
+      <c r="Z7" s="8" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1827,6 +2097,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T8" s="8" t="inlineStr"/>
+      <c r="U8" s="8" t="inlineStr"/>
+      <c r="V8" s="8" t="inlineStr"/>
+      <c r="W8" s="8" t="inlineStr"/>
+      <c r="X8" s="8" t="inlineStr"/>
+      <c r="Y8" s="8" t="inlineStr"/>
+      <c r="Z8" s="8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1910,6 +2187,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T9" s="8" t="inlineStr"/>
+      <c r="U9" s="8" t="inlineStr"/>
+      <c r="V9" s="8" t="inlineStr"/>
+      <c r="W9" s="8" t="inlineStr"/>
+      <c r="X9" s="8" t="inlineStr"/>
+      <c r="Y9" s="8" t="inlineStr"/>
+      <c r="Z9" s="8" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1918,11 +2202,7 @@
 approve</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>PD03 承認管理</t>
-        </is>
-      </c>
+      <c r="B10" s="6" t="inlineStr"/>
       <c r="C10" s="7" t="inlineStr">
         <is>
           <t>◎</t>
@@ -1992,6 +2272,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T10" s="8" t="inlineStr"/>
+      <c r="U10" s="8" t="inlineStr"/>
+      <c r="V10" s="8" t="inlineStr"/>
+      <c r="W10" s="8" t="inlineStr"/>
+      <c r="X10" s="8" t="inlineStr"/>
+      <c r="Y10" s="8" t="inlineStr"/>
+      <c r="Z10" s="8" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2074,6 +2361,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T11" s="8" t="inlineStr"/>
+      <c r="U11" s="8" t="inlineStr"/>
+      <c r="V11" s="8" t="inlineStr"/>
+      <c r="W11" s="8" t="inlineStr"/>
+      <c r="X11" s="8" t="inlineStr"/>
+      <c r="Y11" s="8" t="inlineStr"/>
+      <c r="Z11" s="8" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -2153,6 +2447,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T12" s="8" t="inlineStr"/>
+      <c r="U12" s="8" t="inlineStr"/>
+      <c r="V12" s="8" t="inlineStr"/>
+      <c r="W12" s="8" t="inlineStr"/>
+      <c r="X12" s="8" t="inlineStr"/>
+      <c r="Y12" s="8" t="inlineStr"/>
+      <c r="Z12" s="8" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -2227,6 +2528,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T13" s="8" t="inlineStr"/>
+      <c r="U13" s="8" t="inlineStr"/>
+      <c r="V13" s="8" t="inlineStr"/>
+      <c r="W13" s="8" t="inlineStr"/>
+      <c r="X13" s="8" t="inlineStr"/>
+      <c r="Y13" s="8" t="inlineStr"/>
+      <c r="Z13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2297,6 +2605,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T14" s="8" t="inlineStr"/>
+      <c r="U14" s="8" t="inlineStr"/>
+      <c r="V14" s="8" t="inlineStr"/>
+      <c r="W14" s="8" t="inlineStr"/>
+      <c r="X14" s="8" t="inlineStr"/>
+      <c r="Y14" s="8" t="inlineStr"/>
+      <c r="Z14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -2367,6 +2682,13 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T15" s="8" t="inlineStr"/>
+      <c r="U15" s="8" t="inlineStr"/>
+      <c r="V15" s="8" t="inlineStr"/>
+      <c r="W15" s="8" t="inlineStr"/>
+      <c r="X15" s="8" t="inlineStr"/>
+      <c r="Y15" s="8" t="inlineStr"/>
+      <c r="Z15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2476,17 +2798,24 @@
           <t>RCUDE</t>
         </is>
       </c>
+      <c r="T16" s="8" t="inlineStr"/>
+      <c r="U16" s="8" t="inlineStr"/>
+      <c r="V16" s="8" t="inlineStr"/>
+      <c r="W16" s="8" t="inlineStr"/>
+      <c r="X16" s="8" t="inlineStr"/>
+      <c r="Y16" s="8" t="inlineStr"/>
+      <c r="Z16" s="8" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>社内ドキュメント
-internal_docs</t>
+          <t>管理マニュアル
+admin_manual</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>DC02 社内ドキュメント</t>
+          <t>DC02 管理マニュアル</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -2538,6 +2867,13 @@
         </is>
       </c>
       <c r="S17" s="8" t="inlineStr"/>
+      <c r="T17" s="8" t="inlineStr"/>
+      <c r="U17" s="8" t="inlineStr"/>
+      <c r="V17" s="8" t="inlineStr"/>
+      <c r="W17" s="8" t="inlineStr"/>
+      <c r="X17" s="8" t="inlineStr"/>
+      <c r="Y17" s="8" t="inlineStr"/>
+      <c r="Z17" s="8" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -2548,9 +2884,8 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>SY08 QRカード管理
-SY09 端末管理
-SY0A キオスク設定</t>
+          <t>SY09 端末管理
+SY0A 共有端末設定</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -2574,6 +2909,21 @@
       <c r="Q18" s="8" t="inlineStr"/>
       <c r="R18" s="8" t="inlineStr"/>
       <c r="S18" s="8" t="inlineStr"/>
+      <c r="T18" s="8" t="inlineStr"/>
+      <c r="U18" s="8" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="V18" s="8" t="inlineStr"/>
+      <c r="W18" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="X18" s="8" t="inlineStr"/>
+      <c r="Y18" s="8" t="inlineStr"/>
+      <c r="Z18" s="8" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2584,14 +2934,14 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>SY01 ユーザー管理
-SY02 試算計算
+          <t>SY02 価格試算計算
 SY03 製品項目
 SY04 製品種別
 SY05 アプリ管理
-SY07 操作履歴
 SY0B リンク管理
-SY0C 注文書取込</t>
+SY0C 注文書取込
+SY0E AI プロバイダ
+SY0F 通知メール</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -2615,6 +2965,583 @@
       <c r="Q19" s="8" t="inlineStr"/>
       <c r="R19" s="8" t="inlineStr"/>
       <c r="S19" s="8" t="inlineStr"/>
+      <c r="T19" s="8" t="inlineStr"/>
+      <c r="U19" s="8" t="inlineStr"/>
+      <c r="V19" s="8" t="inlineStr"/>
+      <c r="W19" s="8" t="inlineStr"/>
+      <c r="X19" s="8" t="inlineStr"/>
+      <c r="Y19" s="8" t="inlineStr"/>
+      <c r="Z19" s="8" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>設計図
+design_file</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>PD06 設計図</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>◎</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>RE</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="G20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="H20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr">
+        <is>
+          <t>RCU</t>
+        </is>
+      </c>
+      <c r="K20" s="8" t="inlineStr">
+        <is>
+          <t>RCU</t>
+        </is>
+      </c>
+      <c r="L20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="O20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="Q20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="R20" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="S20" s="8" t="inlineStr">
+        <is>
+          <t>RCUDE</t>
+        </is>
+      </c>
+      <c r="T20" s="8" t="inlineStr"/>
+      <c r="U20" s="8" t="inlineStr"/>
+      <c r="V20" s="8" t="inlineStr"/>
+      <c r="W20" s="8" t="inlineStr"/>
+      <c r="X20" s="8" t="inlineStr"/>
+      <c r="Y20" s="8" t="inlineStr"/>
+      <c r="Z20" s="8" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>フォーム
+form</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr"/>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>◎</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>RE</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr"/>
+      <c r="F21" s="8" t="inlineStr"/>
+      <c r="G21" s="8" t="inlineStr"/>
+      <c r="H21" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I21" s="8" t="inlineStr"/>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr"/>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="inlineStr"/>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="O21" s="8" t="inlineStr"/>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="Q21" s="8" t="inlineStr"/>
+      <c r="R21" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="S21" s="8" t="inlineStr">
+        <is>
+          <t>RCUDE</t>
+        </is>
+      </c>
+      <c r="T21" s="8" t="inlineStr"/>
+      <c r="U21" s="8" t="inlineStr"/>
+      <c r="V21" s="8" t="inlineStr"/>
+      <c r="W21" s="8" t="inlineStr"/>
+      <c r="X21" s="8" t="inlineStr"/>
+      <c r="Y21" s="8" t="inlineStr"/>
+      <c r="Z21" s="8" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>社内文書
+internal_page</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>CM03 社内文書</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>◎</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>RE</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr"/>
+      <c r="F22" s="8" t="inlineStr"/>
+      <c r="G22" s="8" t="inlineStr"/>
+      <c r="H22" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="I22" s="8" t="inlineStr"/>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr"/>
+      <c r="L22" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="inlineStr"/>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="O22" s="8" t="inlineStr"/>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="Q22" s="8" t="inlineStr"/>
+      <c r="R22" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="S22" s="8" t="inlineStr">
+        <is>
+          <t>RCUDE</t>
+        </is>
+      </c>
+      <c r="T22" s="8" t="inlineStr"/>
+      <c r="U22" s="8" t="inlineStr"/>
+      <c r="V22" s="8" t="inlineStr"/>
+      <c r="W22" s="8" t="inlineStr"/>
+      <c r="X22" s="8" t="inlineStr"/>
+      <c r="Y22" s="8" t="inlineStr"/>
+      <c r="Z22" s="8" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>QRカードの発行・PIN
+kiosk_card</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>SY08 QRカード管理</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>◎</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="inlineStr"/>
+      <c r="E23" s="8" t="inlineStr"/>
+      <c r="F23" s="8" t="inlineStr"/>
+      <c r="G23" s="8" t="inlineStr"/>
+      <c r="H23" s="8" t="inlineStr"/>
+      <c r="I23" s="8" t="inlineStr"/>
+      <c r="J23" s="8" t="inlineStr"/>
+      <c r="K23" s="8" t="inlineStr"/>
+      <c r="L23" s="8" t="inlineStr"/>
+      <c r="M23" s="8" t="inlineStr"/>
+      <c r="N23" s="8" t="inlineStr"/>
+      <c r="O23" s="8" t="inlineStr"/>
+      <c r="P23" s="8" t="inlineStr"/>
+      <c r="Q23" s="8" t="inlineStr"/>
+      <c r="R23" s="8" t="inlineStr"/>
+      <c r="S23" s="8" t="inlineStr"/>
+      <c r="T23" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U23" s="8" t="inlineStr">
+        <is>
+          <t>RCU</t>
+        </is>
+      </c>
+      <c r="V23" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W23" s="8" t="inlineStr">
+        <is>
+          <t>RCU</t>
+        </is>
+      </c>
+      <c r="X23" s="8" t="inlineStr"/>
+      <c r="Y23" s="8" t="inlineStr"/>
+      <c r="Z23" s="8" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>端末アクセスの付与
+kiosk_device</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr"/>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>◎</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr"/>
+      <c r="E24" s="8" t="inlineStr"/>
+      <c r="F24" s="8" t="inlineStr"/>
+      <c r="G24" s="8" t="inlineStr"/>
+      <c r="H24" s="8" t="inlineStr"/>
+      <c r="I24" s="8" t="inlineStr"/>
+      <c r="J24" s="8" t="inlineStr"/>
+      <c r="K24" s="8" t="inlineStr"/>
+      <c r="L24" s="8" t="inlineStr"/>
+      <c r="M24" s="8" t="inlineStr"/>
+      <c r="N24" s="8" t="inlineStr"/>
+      <c r="O24" s="8" t="inlineStr"/>
+      <c r="P24" s="8" t="inlineStr"/>
+      <c r="Q24" s="8" t="inlineStr"/>
+      <c r="R24" s="8" t="inlineStr"/>
+      <c r="S24" s="8" t="inlineStr"/>
+      <c r="T24" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U24" s="8" t="inlineStr">
+        <is>
+          <t>RCU</t>
+        </is>
+      </c>
+      <c r="V24" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W24" s="8" t="inlineStr">
+        <is>
+          <t>RCU</t>
+        </is>
+      </c>
+      <c r="X24" s="8" t="inlineStr"/>
+      <c r="Y24" s="8" t="inlineStr"/>
+      <c r="Z24" s="8" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>キオスク端末の秘密
+kiosk_secret</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr"/>
+      <c r="C25" s="7" t="inlineStr">
+        <is>
+          <t>◎</t>
+        </is>
+      </c>
+      <c r="D25" s="8" t="inlineStr"/>
+      <c r="E25" s="8" t="inlineStr"/>
+      <c r="F25" s="8" t="inlineStr"/>
+      <c r="G25" s="8" t="inlineStr"/>
+      <c r="H25" s="8" t="inlineStr"/>
+      <c r="I25" s="8" t="inlineStr"/>
+      <c r="J25" s="8" t="inlineStr"/>
+      <c r="K25" s="8" t="inlineStr"/>
+      <c r="L25" s="8" t="inlineStr"/>
+      <c r="M25" s="8" t="inlineStr"/>
+      <c r="N25" s="8" t="inlineStr"/>
+      <c r="O25" s="8" t="inlineStr"/>
+      <c r="P25" s="8" t="inlineStr"/>
+      <c r="Q25" s="8" t="inlineStr"/>
+      <c r="R25" s="8" t="inlineStr"/>
+      <c r="S25" s="8" t="inlineStr"/>
+      <c r="T25" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="U25" s="8" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="V25" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W25" s="8" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="X25" s="8" t="inlineStr"/>
+      <c r="Y25" s="8" t="inlineStr"/>
+      <c r="Z25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>個人データの閲覧
+personal_data</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>SY07 操作履歴
+SY0D ログイン履歴</t>
+        </is>
+      </c>
+      <c r="C26" s="7" t="inlineStr">
+        <is>
+          <t>◎</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr"/>
+      <c r="E26" s="8" t="inlineStr"/>
+      <c r="F26" s="8" t="inlineStr"/>
+      <c r="G26" s="8" t="inlineStr"/>
+      <c r="H26" s="8" t="inlineStr"/>
+      <c r="I26" s="8" t="inlineStr"/>
+      <c r="J26" s="8" t="inlineStr"/>
+      <c r="K26" s="8" t="inlineStr"/>
+      <c r="L26" s="8" t="inlineStr"/>
+      <c r="M26" s="8" t="inlineStr"/>
+      <c r="N26" s="8" t="inlineStr"/>
+      <c r="O26" s="8" t="inlineStr"/>
+      <c r="P26" s="8" t="inlineStr"/>
+      <c r="Q26" s="8" t="inlineStr"/>
+      <c r="R26" s="8" t="inlineStr"/>
+      <c r="S26" s="8" t="inlineStr"/>
+      <c r="T26" s="8" t="inlineStr"/>
+      <c r="U26" s="8" t="inlineStr"/>
+      <c r="V26" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W26" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="X26" s="8" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="Y26" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z26" s="8" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>取引先ポータルの管理
+portal_admin</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>SY0H 取引先ポータル</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr"/>
+      <c r="D27" s="8" t="inlineStr"/>
+      <c r="E27" s="8" t="inlineStr"/>
+      <c r="F27" s="8" t="inlineStr"/>
+      <c r="G27" s="8" t="inlineStr"/>
+      <c r="H27" s="8" t="inlineStr"/>
+      <c r="I27" s="8" t="inlineStr"/>
+      <c r="J27" s="8" t="inlineStr"/>
+      <c r="K27" s="8" t="inlineStr"/>
+      <c r="L27" s="8" t="inlineStr"/>
+      <c r="M27" s="8" t="inlineStr"/>
+      <c r="N27" s="8" t="inlineStr"/>
+      <c r="O27" s="8" t="inlineStr"/>
+      <c r="P27" s="8" t="inlineStr"/>
+      <c r="Q27" s="8" t="inlineStr"/>
+      <c r="R27" s="8" t="inlineStr"/>
+      <c r="S27" s="8" t="inlineStr"/>
+      <c r="T27" s="8" t="inlineStr"/>
+      <c r="U27" s="8" t="inlineStr"/>
+      <c r="V27" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W27" s="8" t="inlineStr">
+        <is>
+          <t>RCU</t>
+        </is>
+      </c>
+      <c r="X27" s="8" t="inlineStr"/>
+      <c r="Y27" s="8" t="inlineStr"/>
+      <c r="Z27" s="8" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>ユーザー・権限の変更
+user_admin</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>SY01 ユーザー管理</t>
+        </is>
+      </c>
+      <c r="C28" s="7" t="inlineStr">
+        <is>
+          <t>◎</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr"/>
+      <c r="E28" s="8" t="inlineStr"/>
+      <c r="F28" s="8" t="inlineStr"/>
+      <c r="G28" s="8" t="inlineStr"/>
+      <c r="H28" s="8" t="inlineStr"/>
+      <c r="I28" s="8" t="inlineStr"/>
+      <c r="J28" s="8" t="inlineStr"/>
+      <c r="K28" s="8" t="inlineStr"/>
+      <c r="L28" s="8" t="inlineStr"/>
+      <c r="M28" s="8" t="inlineStr"/>
+      <c r="N28" s="8" t="inlineStr"/>
+      <c r="O28" s="8" t="inlineStr"/>
+      <c r="P28" s="8" t="inlineStr"/>
+      <c r="Q28" s="8" t="inlineStr"/>
+      <c r="R28" s="8" t="inlineStr"/>
+      <c r="S28" s="8" t="inlineStr"/>
+      <c r="T28" s="8" t="inlineStr"/>
+      <c r="U28" s="8" t="inlineStr"/>
+      <c r="V28" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="W28" s="8" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="X28" s="8" t="inlineStr"/>
+      <c r="Y28" s="8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="Z28" s="8" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2627,7 +3554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2737,22 +3664,22 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ドキュメント</t>
+          <t>一般</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DC01</t>
+          <t>CM01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>マニュアル</t>
+          <t>承認・予定</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>/manual/ja</t>
+          <t>/general/tasks</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -2765,128 +3692,120 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ドキュメント</t>
+          <t>一般</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DC02</t>
+          <t>CM02</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>社内ドキュメント</t>
+          <t>フォーム</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>/internal-docs/ja</t>
+          <t>/general/forms</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>internal_docs</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>社内ドキュメント</t>
-        </is>
-      </c>
+          <t>（ログインのみ）</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>マスタ</t>
+          <t>一般</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MS01</t>
+          <t>CM03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>取引先</t>
+          <t>社内文書</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>/master/business-partners</t>
+          <t>/general/documents</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>internal_page</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>マスタ管理</t>
+          <t>社内文書</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>マスタ</t>
+          <t>ドキュメント</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MS04</t>
+          <t>DC01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>製品</t>
+          <t>マニュアル</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>/master/products</t>
+          <t>/manual/ja</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>master</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>マスタ管理</t>
-        </is>
-      </c>
+          <t>（ログインのみ）</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>マスタ</t>
+          <t>ドキュメント</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MS05</t>
+          <t>DC02</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>材種</t>
+          <t>管理マニュアル</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>/master/material-types</t>
+          <t>/admin-manual/ja</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>master</t>
+          <t>admin_manual</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>マスタ管理</t>
+          <t>管理マニュアル</t>
         </is>
       </c>
     </row>
@@ -2898,17 +3817,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MS06</t>
+          <t>MS01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>素材</t>
+          <t>取引先</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>/master/materials</t>
+          <t>/master/business-partners</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -2930,17 +3849,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MS07</t>
+          <t>MS04</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>採番構成</t>
+          <t>製品</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>/master/material-numbering</t>
+          <t>/master/products</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -2962,17 +3881,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MS08</t>
+          <t>MS05</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>工程マスタ</t>
+          <t>材種</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>/master/process-steps</t>
+          <t>/master/material-types</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -2994,17 +3913,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>MS09</t>
+          <t>MS06</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>検査表テンプレート</t>
+          <t>素材</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>/master/inspection-templates</t>
+          <t>/master/materials</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -3026,17 +3945,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MS0A</t>
+          <t>MS07</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>不良種類</t>
+          <t>採番構成</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>/master/defect-types</t>
+          <t>/master/material-numbering</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3058,17 +3977,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MS0B</t>
+          <t>MS08</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>承認設定</t>
+          <t>工程マスタ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>/master/approval-settings</t>
+          <t>/master/process-steps</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -3090,17 +4009,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MS0C</t>
+          <t>MS09</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>拠点</t>
+          <t>検査表テンプレート</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>/master/plants</t>
+          <t>/master/inspection-templates</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3122,17 +4041,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MS0D</t>
+          <t>MS0A</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>作業場所</t>
+          <t>不良種類</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>/master/work-locations</t>
+          <t>/master/defect-types</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3154,17 +4073,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>MS0E</t>
+          <t>MS0B</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>保管場所</t>
+          <t>承認設定</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>/master/storage-locations</t>
+          <t>/master/approval-settings</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3181,96 +4100,96 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>生産</t>
+          <t>マスタ</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>PD02</t>
+          <t>MS0C</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>指示書</t>
+          <t>拠点</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>/production/work-orders</t>
+          <t>/master/plants</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>work_order</t>
+          <t>master</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>指示書</t>
+          <t>マスタ管理</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>生産</t>
+          <t>マスタ</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>PD03</t>
+          <t>MS0D</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>承認管理</t>
+          <t>作業場所</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>/production/approvals</t>
+          <t>/master/work-locations</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>approve</t>
+          <t>master</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>承認管理</t>
+          <t>マスタ管理</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>生産</t>
+          <t>マスタ</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>PD04</t>
+          <t>MS0E</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>在庫管理</t>
+          <t>保管場所</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>/production/inventory</t>
+          <t>/master/storage-locations</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>inventory</t>
+          <t>master</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>在庫</t>
+          <t>マスタ管理</t>
         </is>
       </c>
     </row>
@@ -3282,17 +4201,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PD05</t>
+          <t>PD02</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>未処理指示書</t>
+          <t>指示書</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>/production/pending-work-orders</t>
+          <t>/production/work-orders</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3309,96 +4228,96 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>購買</t>
+          <t>生産</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PU01</t>
+          <t>PD04</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>購買依頼</t>
+          <t>在庫管理</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>/purchase/purchase-requests</t>
+          <t>/production/inventory</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>purchase_order</t>
+          <t>inventory</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>素材発注・購買依頼</t>
+          <t>在庫</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>購買</t>
+          <t>生産</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>PU02</t>
+          <t>PD05</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>素材発注書</t>
+          <t>未処理指示書</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>/purchase/purchase-orders</t>
+          <t>/production/pending-work-orders</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>purchase_order</t>
+          <t>work_order</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>素材発注・購買依頼</t>
+          <t>指示書</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>購買</t>
+          <t>生産</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>PU03</t>
+          <t>PD06</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>素材入荷</t>
+          <t>設計図</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>/purchase/material-receipts</t>
+          <t>/production/design-files</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>material_receipt</t>
+          <t>design_file</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>素材入荷</t>
+          <t>設計図</t>
         </is>
       </c>
     </row>
@@ -3410,123 +4329,123 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PU04</t>
+          <t>PU01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>外注依頼</t>
+          <t>購買依頼</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>/purchase/outsource-orders</t>
+          <t>/purchase/purchase-requests</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>outsource_order</t>
+          <t>purchase_order</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>外注依頼</t>
+          <t>素材発注・購買依頼</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>販売</t>
+          <t>購買</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SA01</t>
+          <t>PU02</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>試算</t>
+          <t>素材発注書</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>/sales/trial-estimates</t>
+          <t>/purchase/purchase-orders</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>price_list</t>
+          <t>purchase_order</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>価格表</t>
+          <t>素材発注・購買依頼</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>販売</t>
+          <t>購買</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SA02</t>
+          <t>PU03</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>価格表</t>
+          <t>素材入荷</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>/sales/price-lists</t>
+          <t>/purchase/material-receipts</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>price_list</t>
+          <t>material_receipt</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>価格表</t>
+          <t>素材入荷</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>販売</t>
+          <t>購買</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SA03</t>
+          <t>PU04</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>見積書</t>
+          <t>外注依頼</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>/sales/quotes</t>
+          <t>/purchase/outsource-orders</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>quote</t>
+          <t>outsource_order</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>見積書</t>
+          <t>外注依頼</t>
         </is>
       </c>
     </row>
@@ -3538,27 +4457,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SA04</t>
+          <t>SA01</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>注文請書</t>
+          <t>価格試算</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>/sales/order-acceptances</t>
+          <t>/sales/trial-estimates</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>order_acceptance</t>
+          <t>price_list</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>受注請書・受注明細</t>
+          <t>価格表</t>
         </is>
       </c>
     </row>
@@ -3570,27 +4489,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>SA05</t>
+          <t>SA02</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>注文明細</t>
+          <t>価格表</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>/sales/order-lines</t>
+          <t>/sales/price-lists</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>order_acceptance</t>
+          <t>price_list</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>受注請書・受注明細</t>
+          <t>価格表</t>
         </is>
       </c>
     </row>
@@ -3602,219 +4521,219 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>SA06</t>
+          <t>SA03</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>設計依頼書</t>
+          <t>見積書</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>/sales/design-requests</t>
+          <t>/sales/quotes</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>design_request</t>
+          <t>quote</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>設計依頼</t>
+          <t>見積書</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>出荷</t>
+          <t>販売</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>SH01</t>
+          <t>SA04</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>出荷書</t>
+          <t>注文請書</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>/shipping/delivery-orders</t>
+          <t>/sales/order-acceptances</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>delivery_order</t>
+          <t>order_acceptance</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>出荷書</t>
+          <t>受注請書・受注明細</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>出荷</t>
+          <t>販売</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>SH02</t>
+          <t>SA05</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>納品書</t>
+          <t>注文明細</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>/shipping/delivery-notes</t>
+          <t>/sales/order-lines</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>delivery_note</t>
+          <t>order_acceptance</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>納品書</t>
+          <t>受注請書・受注明細</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>出荷</t>
+          <t>販売</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>SH03</t>
+          <t>SA06</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>未処理出荷書</t>
+          <t>設計依頼書</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>/shipping/pending-shipments</t>
+          <t>/sales/design-requests</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>delivery_order</t>
+          <t>design_request</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>出荷書</t>
+          <t>設計依頼</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>システム</t>
+          <t>出荷</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>SY01</t>
+          <t>SH01</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>ユーザー管理</t>
+          <t>出荷書</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>/settings/users</t>
+          <t>/shipping/delivery-orders</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>delivery_order</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>システム管理</t>
+          <t>出荷書</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>システム</t>
+          <t>出荷</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>SY02</t>
+          <t>SH02</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>試算計算</t>
+          <t>納品書</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>/settings/trial-pricing-engine</t>
+          <t>/shipping/delivery-notes</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>delivery_note</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>システム管理</t>
+          <t>納品書</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>システム</t>
+          <t>出荷</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>SY03</t>
+          <t>SH03</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>製品項目</t>
+          <t>未処理出荷書</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>/settings/product-items</t>
+          <t>/shipping/pending-shipments</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>delivery_order</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>システム管理</t>
+          <t>出荷書</t>
         </is>
       </c>
     </row>
@@ -3826,27 +4745,27 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>SY04</t>
+          <t>SY01</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>製品種別</t>
+          <t>ユーザー管理</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>/settings/product-types</t>
+          <t>/settings/users</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>user_admin</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>システム管理</t>
+          <t>ユーザー・権限の変更</t>
         </is>
       </c>
     </row>
@@ -3858,17 +4777,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SY05</t>
+          <t>SY02</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>アプリ管理</t>
+          <t>価格試算計算</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>/settings/apps</t>
+          <t>/settings/trial-pricing-engine</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -3890,25 +4809,29 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>SY06</t>
+          <t>SY03</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ファイル管理</t>
+          <t>製品項目</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>/settings/files</t>
+          <t>/settings/product-items</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>（ログインのみ）</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>システム管理</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3918,17 +4841,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SY07</t>
+          <t>SY04</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>操作履歴</t>
+          <t>製品種別</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>/settings/activity</t>
+          <t>/settings/product-types</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -3950,27 +4873,27 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>SY08</t>
+          <t>SY05</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>QRカード管理</t>
+          <t>アプリ管理</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>/settings/kiosk-cards</t>
+          <t>/settings/apps</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>kiosk</t>
+          <t>system</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>キオスク管理</t>
+          <t>システム管理</t>
         </is>
       </c>
     </row>
@@ -3982,29 +4905,25 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>SY09</t>
+          <t>SY06</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>端末管理</t>
+          <t>ファイル管理</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>/settings/kiosk-devices</t>
+          <t>/settings/files</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>kiosk</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>キオスク管理</t>
-        </is>
-      </c>
+          <t>（ログインのみ）</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4014,27 +4933,27 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>SY0A</t>
+          <t>SY07</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>キオスク設定</t>
+          <t>操作履歴</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>/settings/kiosk</t>
+          <t>/settings/activity</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>kiosk</t>
+          <t>personal_data</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>キオスク管理</t>
+          <t>個人データの閲覧</t>
         </is>
       </c>
     </row>
@@ -4046,27 +4965,27 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SY0B</t>
+          <t>SY08</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>リンク管理</t>
+          <t>QRカード管理</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>/settings/links</t>
+          <t>/settings/kiosk-cards</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>kiosk_card</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>システム管理</t>
+          <t>QRカードの発行・PIN</t>
         </is>
       </c>
     </row>
@@ -4078,27 +4997,279 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>SY09</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>端末管理</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>/settings/kiosk-devices</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>kiosk</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>キオスク管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>SY0A</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>共有端末設定</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>/settings/kiosk</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>kiosk</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>キオスク管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>SY0B</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>リンク管理</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>/settings/links</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>システム管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
           <t>SY0C</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>注文書取込</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>/settings/order-intake</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>システム管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>SY0D</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ログイン履歴</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>/settings/login-history</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>personal_data</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>個人データの閲覧</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>SY0E</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>AI プロバイダ</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>/settings/ai-provider</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>システム管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>SY0F</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>通知メール</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>/settings/notification-email</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>システム管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>SY0G</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>特権アクセス</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>/settings/privileged-access</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>（ログインのみ）</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>SY0H</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>取引先ポータル</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>/settings/portal</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>portal_admin</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>取引先ポータルの管理</t>
         </is>
       </c>
     </row>
@@ -4113,7 +5284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4159,12 +5330,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>demo1</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>田中 一郎（管理）</t>
+          <t>管理者</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -4177,31 +5348,27 @@
           <t>○</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>demo2026</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>SSO / 実ユーザー</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>demo2</t>
+          <t>demo1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>鈴木 二郎（営業）</t>
+          <t>田中 一郎（管理）</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>staff</t>
+          <t>admin</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4216,19 +5383,19 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>demo3</t>
+          <t>demo2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>佐藤 三郎（製造）</t>
+          <t>鈴木 二郎（営業）</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -4248,19 +5415,19 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>demo4</t>
+          <t>demo3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>高橋 四子（検査）</t>
+          <t>佐藤 三郎（製造）</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4280,19 +5447,19 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>demo5</t>
+          <t>demo4</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>伊藤 五月（出荷）</t>
+          <t>高橋 四子（検査）</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -4312,24 +5479,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>dev_accounting</t>
+          <t>demo5</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>開発 経理</t>
+          <t>伊藤 五月（出荷）</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>accounting</t>
+          <t>staff</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4339,29 +5506,29 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>dev2026</t>
+          <t>demo2026</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>dev_accounting_mgr</t>
+          <t>dev_accounting</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>開発 経理部長</t>
+          <t>開発 経理</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>accounting_manager</t>
+          <t>accounting</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4376,24 +5543,24 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>dev_manager</t>
+          <t>dev_accounting_mgr</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>開発 管理職</t>
+          <t>開発 経理部長</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>manager</t>
+          <t>accounting_manager</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -4408,24 +5575,24 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dev_production</t>
+          <t>dev_manager</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>開発 製造</t>
+          <t>開発 管理職</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>production</t>
+          <t>manager</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -4440,24 +5607,24 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dev_production_mgr</t>
+          <t>dev_production</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>開発 製造部長</t>
+          <t>開発 製造</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>production_manager</t>
+          <t>production</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -4472,24 +5639,24 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dev_purchasing</t>
+          <t>dev_production_mgr</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>開発 購買</t>
+          <t>開発 製造部長</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>purchasing</t>
+          <t>production_manager</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -4504,24 +5671,24 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>dev_purchasing_mgr</t>
+          <t>dev_purchasing</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>開発 購買部長</t>
+          <t>開発 購買</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>purchasing_manager</t>
+          <t>purchasing</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -4536,24 +5703,24 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>dev_quality</t>
+          <t>dev_purchasing_mgr</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>開発 品質</t>
+          <t>開発 購買部長</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>quality</t>
+          <t>purchasing_manager</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -4568,24 +5735,24 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dev_quality_mgr</t>
+          <t>dev_quality</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>開発 品質部長</t>
+          <t>開発 品質</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>quality_manager</t>
+          <t>quality</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -4600,24 +5767,24 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>dev_sales</t>
+          <t>dev_quality_mgr</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>開発 営業</t>
+          <t>開発 品質部長</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>sales</t>
+          <t>quality_manager</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -4632,24 +5799,24 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dev_sales_assistant</t>
+          <t>dev_sales</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>開発 営業補佐</t>
+          <t>開発 営業</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sales_assistant</t>
+          <t>sales</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -4664,24 +5831,24 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>dev_sales_mgr</t>
+          <t>dev_sales_assistant</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>開発 営業部長</t>
+          <t>開発 営業補佐</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>sales_manager</t>
+          <t>sales_assistant</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -4696,24 +5863,24 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>dev_shipping</t>
+          <t>dev_sales_mgr</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>開発 出荷</t>
+          <t>開発 営業部長</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>sales_manager</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -4728,24 +5895,24 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>dev_shipping_mgr</t>
+          <t>dev_shipping</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>開発 出荷部長</t>
+          <t>開発 出荷</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>shipping_manager</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -4760,24 +5927,24 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>dev_viewer</t>
+          <t>dev_shipping_mgr</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>開発 閲覧</t>
+          <t>開発 出荷部長</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>viewer</t>
+          <t>shipping_manager</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -4792,24 +5959,24 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>ckk-dev.kai-lab.net（検証専用）</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>k.sawada</t>
+          <t>dev_viewer</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>澤田 魁星</t>
+          <t>開発 閲覧</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>（未割当）</t>
+          <t>viewer</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -4817,22 +5984,26 @@
           <t>○</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>dev2026</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>SSO / 実ユーザー</t>
+          <t>app-dev.ckk-tool.co.jp（検証専用）</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>system</t>
+          <t>k.sawada</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>システム</t>
+          <t>澤田 魁星</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -4847,6 +6018,34 @@
       </c>
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
+        <is>
+          <t>SSO / 実ユーザー</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>system</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>システム</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>（未割当）</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>○</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
         <is>
           <t>SSO / 実ユーザー</t>
         </is>

</xml_diff>